<commit_message>
Fixed the all product and portfollio tests
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="180">
   <si>
     <t xml:space="preserve">TestCase</t>
   </si>
@@ -473,6 +473,93 @@
   </si>
   <si>
     <t>validateMyProductPortfolios</t>
+  </si>
+  <si>
+    <t>AddTeamsAndMembersToProduct</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260924_182820_023</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260924_182820_023: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260924_183147_837</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260924_183147_837: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_102912_743</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_102912_743: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_103413_199</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_103413_199: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_120815_652</t>
+  </si>
+  <si>
+    <t>Automation Private Team Allocation Product_20260925_120815_652: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>AddProductToRelease</t>
+  </si>
+  <si>
+    <t>Automation Private Release Product_20260928_081923_317</t>
+  </si>
+  <si>
+    <t>Automation Private Release Product_20260928_081923_317: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Digital_20260928_081901_818</t>
+  </si>
+  <si>
+    <t>Digital Platform Hotfix_20260928_081912_145</t>
+  </si>
+  <si>
+    <t>ValidationOfCustomFields</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20260928_152816_158</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20260928_152816_158: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Public Custom Fields Product_20260928_164703_453</t>
+  </si>
+  <si>
+    <t>Automation Public Custom Fields Product_20260928_164703_453: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Public Custom Fields Product_20260928_165734_283</t>
+  </si>
+  <si>
+    <t>Automation Public Custom Fields Product_20260928_165734_283: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>downloadAuditHistoryInPdfAndCsvFormats</t>
+  </si>
+  <si>
+    <t>Automation Report Portfolio_20260928_170613_206</t>
+  </si>
+  <si>
+    <t>Automation Report Portfolio_20260928_170948_480</t>
+  </si>
+  <si>
+    <t>Automation Report Portfolio_20260928_172347_502</t>
+  </si>
+  <si>
+    <t>Automation Report Portfolio_20260928_172732_811</t>
+  </si>
+  <si>
+    <t>Automation Report Portfolio_20260928_172939_485</t>
   </si>
 </sst>
 </file>
@@ -762,7 +849,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" customWidth="true" hidden="false" style="0" width="27.15" collapsed="false" outlineLevel="0"/>
@@ -1715,6 +1802,170 @@
         <v>21</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>151</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>161</v>
+      </c>
+      <c r="F24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="H24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="J24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="L24" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="M24" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>162</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>163</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>164</v>
+      </c>
+      <c r="F25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="H25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="J25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K25" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="L25" t="s" s="0">
+        <v>165</v>
+      </c>
+      <c r="M25" t="s" s="0">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="0">
+        <v>167</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>109</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="F26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="H26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="J26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="L26" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="M26" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="C27" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="H27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="J27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="L27" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="M27" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added 11th test case
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="184">
   <si>
     <t xml:space="preserve">TestCase</t>
   </si>
@@ -560,6 +560,18 @@
   </si>
   <si>
     <t>Automation Report Portfolio_20260928_172939_485</t>
+  </si>
+  <si>
+    <t>EditPortfolioDetailsOfExistingProduct</t>
+  </si>
+  <si>
+    <t>Updated Existing Product Portfolio_20260929_132500_259</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_132436_044</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_132436_044: Define, Design, Develop, Deploy</t>
   </si>
 </sst>
 </file>
@@ -849,7 +861,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" customWidth="true" hidden="false" style="0" width="27.15" collapsed="false" outlineLevel="0"/>
@@ -1966,6 +1978,47 @@
         <v>21</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="s" s="0">
+        <v>180</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>181</v>
+      </c>
+      <c r="C28" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>182</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>183</v>
+      </c>
+      <c r="F28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="H28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="J28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="L28" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="M28" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
11th test case fix
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="193">
   <si>
     <t xml:space="preserve">TestCase</t>
   </si>
@@ -572,6 +572,33 @@
   </si>
   <si>
     <t>Automation Product_20260929_132436_044: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Updated Existing Product Portfolio_20260929_135503_976</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_135439_778</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_135439_778: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Updated Existing Product Portfolio_20260929_135939_935</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_135910_097</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_135910_097: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Updated Existing Product Portfolio_20260929_140454_551</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_140429_742</t>
+  </si>
+  <si>
+    <t>Automation Product_20260929_140429_742: Define, Design, Develop, Deploy</t>
   </si>
 </sst>
 </file>
@@ -1983,16 +2010,16 @@
         <v>180</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="C28" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="F28" t="s" s="0">
         <v>21</v>

</xml_diff>

<commit_message>
Added the new test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -6,12 +6,13 @@
   </bookViews>
   <sheets>
     <sheet name="ProE2E" sheetId="1" r:id="rId4"/>
+    <sheet name="MaturityAssessments" r:id="rId5" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="211" count="1045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="224" count="1063">
   <si>
     <t>TestCase</t>
   </si>
@@ -644,6 +645,45 @@
   </si>
   <si>
     <t>Automation Public Product_20261015_144937_631: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>AssessmentName</t>
+  </si>
+  <si>
+    <t>MaturityAssesmentAtOrganisationLevel</t>
+  </si>
+  <si>
+    <t>Organization Automation and AI Readiness_20261020_195258_768</t>
+  </si>
+  <si>
+    <t>Organization Automation and AI Readiness_20261020_200619_684</t>
+  </si>
+  <si>
+    <t>MaturityAssesmentOrganisationRespondToAssesement</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_095352_404</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_101536_356</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_102226_124</t>
+  </si>
+  <si>
+    <t>IntiateAndDiscardMaturityAssessmentAtOrgLevel</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_151013_455</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_151149_527</t>
+  </si>
+  <si>
+    <t>BaseLineOrganisationMaturtiyAssesement</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261021_163036_437</t>
   </si>
 </sst>
 </file>
@@ -2887,4 +2927,54 @@
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>215</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>222</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>223</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed time zone issue
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="292" count="1415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="296" count="1439">
   <si>
     <t>TestCase</t>
   </si>
@@ -888,6 +888,18 @@
   </si>
   <si>
     <t>Automation Product_20261022_191858_071: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20261023_115746_432</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20261023_115746_432: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20261023_121205_351</t>
+  </si>
+  <si>
+    <t>Automation Public Product_20261023_121205_351: Define, Design, Develop, Deploy</t>
   </si>
 </sst>
 </file>
@@ -2807,10 +2819,10 @@
         <v>15</v>
       </c>
       <c r="D19" t="s" s="1">
-        <v>209</v>
+        <v>294</v>
       </c>
       <c r="E19" t="s" s="1">
-        <v>210</v>
+        <v>295</v>
       </c>
       <c r="F19" t="s" s="1">
         <v>15</v>

</xml_diff>

<commit_message>
Added the 2 more cases
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="296" count="1439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="310" count="1503">
   <si>
     <t>TestCase</t>
   </si>
@@ -900,6 +900,48 @@
   </si>
   <si>
     <t>Automation Public Product_20261023_121205_351: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Product_20261023_123333_433</t>
+  </si>
+  <si>
+    <t>Automation Product_20261023_123333_433: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Product_20261023_123745_886</t>
+  </si>
+  <si>
+    <t>Automation Product_20261023_123745_886: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Product_20261023_123745_886: Automation Linked Feature For Deletion_20261023_123829_023</t>
+  </si>
+  <si>
+    <t>Automation Linked Feature For Deletion_20261023_123829_023: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>MaturityAssessmentCompletedAssessmentValidation</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261023_124428_879</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261023_124428_879: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>SaveMaturityAssessmentWithoutSubmittingAndVerifyResume</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261023_140053_384</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261023_140053_384: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>MaturityAssesmentAtOrganisationValidateInitiateOption</t>
+  </si>
+  <si>
+    <t>Org Maturity_20261023_152034_621</t>
   </si>
 </sst>
 </file>
@@ -2056,7 +2098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="27.1719"/>
@@ -2204,10 +2246,10 @@
         <v>15</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="F4" t="s" s="1">
         <v>15</v>
@@ -2245,16 +2287,16 @@
         <v>15</v>
       </c>
       <c r="D5" t="s" s="1">
-        <v>120</v>
+        <v>298</v>
       </c>
       <c r="E5" t="s" s="1">
-        <v>121</v>
+        <v>299</v>
       </c>
       <c r="F5" t="s" s="1">
-        <v>122</v>
+        <v>300</v>
       </c>
       <c r="G5" t="s" s="1">
-        <v>123</v>
+        <v>301</v>
       </c>
       <c r="H5" t="s" s="1">
         <v>15</v>
@@ -3461,6 +3503,88 @@
         <v>15</v>
       </c>
       <c r="M34" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="1">
+        <v>302</v>
+      </c>
+      <c r="B35" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="C35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="D35" t="s" s="1">
+        <v>303</v>
+      </c>
+      <c r="E35" t="s" s="1">
+        <v>304</v>
+      </c>
+      <c r="F35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="I35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="J35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="K35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="L35" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="M35" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="1">
+        <v>305</v>
+      </c>
+      <c r="B36" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="C36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="D36" t="s" s="1">
+        <v>306</v>
+      </c>
+      <c r="E36" t="s" s="1">
+        <v>307</v>
+      </c>
+      <c r="F36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="I36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="J36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="K36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="L36" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="M36" t="s" s="1">
         <v>15</v>
       </c>
     </row>
@@ -3475,7 +3599,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3518,6 +3642,14 @@
         <v>224</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>309</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added 8 more test cases
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="310" count="1503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="331" count="1614">
   <si>
     <t>TestCase</t>
   </si>
@@ -942,6 +942,69 @@
   </si>
   <si>
     <t>Org Maturity_20261023_152034_621</t>
+  </si>
+  <si>
+    <t>VerifyBaselinedAssessmentsSearchByProductNameAtProdcutLevel</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_104630_503</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_104630_503: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>VerifyCurrentAssessmentsSearchByProductNameAtProdcutLevel</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_111157_171</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_111157_171: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_123321_665</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_123321_665: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_124142_037</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_124142_037: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_125210_988</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_125210_988: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_130655_236</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_130655_236: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_131216_927</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_131216_927: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_131622_454</t>
+  </si>
+  <si>
+    <t>Automation Private Product Maturity Assessment_20261027_131622_454: Define, Design, Develop, Deploy</t>
+  </si>
+  <si>
+    <t>VerifyCurrentAssessmentsSearchByTeamNameAtTeamLevel</t>
+  </si>
+  <si>
+    <t>Automation Private Product Team Maturity Assessment_20261027_210639_946</t>
+  </si>
+  <si>
+    <t>Automation Private Product Team Maturity Assessment_20261027_210639_946: Define, Design, Develop, Deploy</t>
   </si>
 </sst>
 </file>
@@ -2098,7 +2161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultColWidth="8.5" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" customWidth="true" style="1" width="27.1719"/>
@@ -3585,6 +3648,129 @@
         <v>15</v>
       </c>
       <c r="M36" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="1">
+        <v>310</v>
+      </c>
+      <c r="B37" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="C37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="D37" t="s" s="1">
+        <v>320</v>
+      </c>
+      <c r="E37" t="s" s="1">
+        <v>321</v>
+      </c>
+      <c r="F37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="I37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="J37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="K37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="L37" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="M37" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="1">
+        <v>313</v>
+      </c>
+      <c r="B38" t="s" s="1">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="D38" t="s" s="1">
+        <v>326</v>
+      </c>
+      <c r="E38" t="s" s="1">
+        <v>327</v>
+      </c>
+      <c r="F38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="I38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="J38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="K38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="L38" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="M38" t="s" s="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="1">
+        <v>328</v>
+      </c>
+      <c r="B39" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="C39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="D39" t="s" s="1">
+        <v>329</v>
+      </c>
+      <c r="E39" t="s" s="1">
+        <v>330</v>
+      </c>
+      <c r="F39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="G39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="I39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="J39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="K39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="L39" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="M39" t="s" s="1">
         <v>15</v>
       </c>
     </row>

</xml_diff>